<commit_message>
:feet 칼만필터 seed값 고정 update
</commit_message>
<xml_diff>
--- a/칼만필터_ex.xlsx
+++ b/칼만필터_ex.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python\Kalman_Filter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45DBA9DF-E0DA-4DA8-8B39-4C660EB3174A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76EDE227-F2AE-450B-8B03-EE1D8B2C13CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{1D83DCE4-FA4F-4273-B006-597E1AD51264}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -465,7 +465,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>53.206000000000003</v>
+        <v>50.993000000000002</v>
       </c>
       <c r="C3">
         <v>50</v>
@@ -489,7 +489,7 @@
       </c>
       <c r="I3">
         <f>C3+H3*(B3-C3)</f>
-        <v>51.603200349956253</v>
+        <v>50.496562054743158</v>
       </c>
       <c r="J3">
         <f>(1-H3)*G3</f>
@@ -501,11 +501,11 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>48.982999999999997</v>
+        <v>49.722999999999999</v>
       </c>
       <c r="C4">
         <f>I3</f>
-        <v>51.603200349956253</v>
+        <v>50.496562054743158</v>
       </c>
       <c r="D4">
         <v>1E-3</v>
@@ -527,7 +527,7 @@
       </c>
       <c r="I4">
         <f>C4+H4*(B4-C4)</f>
-        <v>50.729436401482076</v>
+        <v>50.23860062238419</v>
       </c>
       <c r="J4">
         <f>(1-H4)*G4</f>
@@ -539,11 +539,11 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>49.944000000000003</v>
+        <v>51.295000000000002</v>
       </c>
       <c r="C5">
         <f>I4</f>
-        <v>50.729436401482076</v>
+        <v>50.23860062238419</v>
       </c>
       <c r="D5">
         <v>1E-3</v>
@@ -565,7 +565,7 @@
       </c>
       <c r="I5">
         <f>C5+H5*(B5-C5)</f>
-        <v>50.532905551302612</v>
+        <v>50.502931467529812</v>
       </c>
       <c r="J5">
         <f>(1-H5)*G5</f>

</xml_diff>